<commit_message>
update code: 09/14/2025. Phase 1 complete - python code
</commit_message>
<xml_diff>
--- a/nba_described01.xlsx
+++ b/nba_described01.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10830"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oaitran/Desktop/PhD/Fall_2025/DS_7200/final_project/DS_7200_final_project/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08417F9-8AC7-D24B-BA00-556815D15C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="122">
   <si>
     <t>player_total</t>
   </si>
@@ -169,148 +163,151 @@
     <t>2TM</t>
   </si>
   <si>
+    <t>PF</t>
+  </si>
+  <si>
+    <t>player_Award_Shares</t>
+  </si>
+  <si>
+    <t>award</t>
+  </si>
+  <si>
+    <t>first</t>
+  </si>
+  <si>
+    <t>pts_won</t>
+  </si>
+  <si>
+    <t>pts_max</t>
+  </si>
+  <si>
+    <t>share</t>
+  </si>
+  <si>
+    <t>winner</t>
+  </si>
+  <si>
+    <t>nba mip</t>
+  </si>
+  <si>
+    <t>LeBron James</t>
+  </si>
+  <si>
+    <t>jamesle01</t>
+  </si>
+  <si>
+    <t>player_per_game</t>
+  </si>
+  <si>
+    <t>mp_per_game</t>
+  </si>
+  <si>
+    <t>fg_per_game</t>
+  </si>
+  <si>
+    <t>fga_per_game</t>
+  </si>
+  <si>
+    <t>x3p_per_game</t>
+  </si>
+  <si>
+    <t>x3pa_per_game</t>
+  </si>
+  <si>
+    <t>x2p_per_game</t>
+  </si>
+  <si>
+    <t>x2pa_per_game</t>
+  </si>
+  <si>
+    <t>ft_per_game</t>
+  </si>
+  <si>
+    <t>fta_per_game</t>
+  </si>
+  <si>
+    <t>orb_per_game</t>
+  </si>
+  <si>
+    <t>drb_per_game</t>
+  </si>
+  <si>
+    <t>trb_per_game</t>
+  </si>
+  <si>
+    <t>ast_per_game</t>
+  </si>
+  <si>
+    <t>stl_per_game</t>
+  </si>
+  <si>
+    <t>blk_per_game</t>
+  </si>
+  <si>
+    <t>tov_per_game</t>
+  </si>
+  <si>
+    <t>pf_per_game</t>
+  </si>
+  <si>
+    <t>pts_per_game</t>
+  </si>
+  <si>
+    <t>player_play_by_play</t>
+  </si>
+  <si>
+    <t>pg_percent</t>
+  </si>
+  <si>
+    <t>sg_percent</t>
+  </si>
+  <si>
+    <t>sf_percent</t>
+  </si>
+  <si>
+    <t>pf_percent</t>
+  </si>
+  <si>
+    <t>c_percent</t>
+  </si>
+  <si>
+    <t>on_court_plus_minus_per_100_poss</t>
+  </si>
+  <si>
+    <t>net_plus_minus_per_100_poss</t>
+  </si>
+  <si>
+    <t>bad_pass_turnover</t>
+  </si>
+  <si>
+    <t>lost_ball_turnover</t>
+  </si>
+  <si>
+    <t>shooting_foul_committed</t>
+  </si>
+  <si>
+    <t>offensive_foul_committed</t>
+  </si>
+  <si>
+    <t>shooting_foul_drawn</t>
+  </si>
+  <si>
+    <t>offensive_foul_drawn</t>
+  </si>
+  <si>
+    <t>points_generated_by_assists</t>
+  </si>
+  <si>
+    <t>and1</t>
+  </si>
+  <si>
+    <t>fga_blocked</t>
+  </si>
+  <si>
+    <t>Nazr Mohammed</t>
+  </si>
+  <si>
     <t>SG</t>
-  </si>
-  <si>
-    <t>player_Award_Shares</t>
-  </si>
-  <si>
-    <t>award</t>
-  </si>
-  <si>
-    <t>first</t>
-  </si>
-  <si>
-    <t>pts_won</t>
-  </si>
-  <si>
-    <t>pts_max</t>
-  </si>
-  <si>
-    <t>share</t>
-  </si>
-  <si>
-    <t>winner</t>
-  </si>
-  <si>
-    <t>nba mvp</t>
-  </si>
-  <si>
-    <t>LeBron James</t>
-  </si>
-  <si>
-    <t>jamesle01</t>
-  </si>
-  <si>
-    <t>player_per_game</t>
-  </si>
-  <si>
-    <t>mp_per_game</t>
-  </si>
-  <si>
-    <t>fg_per_game</t>
-  </si>
-  <si>
-    <t>fga_per_game</t>
-  </si>
-  <si>
-    <t>x3p_per_game</t>
-  </si>
-  <si>
-    <t>x3pa_per_game</t>
-  </si>
-  <si>
-    <t>x2p_per_game</t>
-  </si>
-  <si>
-    <t>x2pa_per_game</t>
-  </si>
-  <si>
-    <t>ft_per_game</t>
-  </si>
-  <si>
-    <t>fta_per_game</t>
-  </si>
-  <si>
-    <t>orb_per_game</t>
-  </si>
-  <si>
-    <t>drb_per_game</t>
-  </si>
-  <si>
-    <t>trb_per_game</t>
-  </si>
-  <si>
-    <t>ast_per_game</t>
-  </si>
-  <si>
-    <t>stl_per_game</t>
-  </si>
-  <si>
-    <t>blk_per_game</t>
-  </si>
-  <si>
-    <t>tov_per_game</t>
-  </si>
-  <si>
-    <t>pf_per_game</t>
-  </si>
-  <si>
-    <t>pts_per_game</t>
-  </si>
-  <si>
-    <t>player_play_by_play</t>
-  </si>
-  <si>
-    <t>pg_percent</t>
-  </si>
-  <si>
-    <t>sg_percent</t>
-  </si>
-  <si>
-    <t>sf_percent</t>
-  </si>
-  <si>
-    <t>pf_percent</t>
-  </si>
-  <si>
-    <t>c_percent</t>
-  </si>
-  <si>
-    <t>on_court_plus_minus_per_100_poss</t>
-  </si>
-  <si>
-    <t>net_plus_minus_per_100_poss</t>
-  </si>
-  <si>
-    <t>bad_pass_turnover</t>
-  </si>
-  <si>
-    <t>lost_ball_turnover</t>
-  </si>
-  <si>
-    <t>shooting_foul_committed</t>
-  </si>
-  <si>
-    <t>offensive_foul_committed</t>
-  </si>
-  <si>
-    <t>shooting_foul_drawn</t>
-  </si>
-  <si>
-    <t>offensive_foul_drawn</t>
-  </si>
-  <si>
-    <t>points_generated_by_assists</t>
-  </si>
-  <si>
-    <t>and1</t>
-  </si>
-  <si>
-    <t>fga_blocked</t>
-  </si>
-  <si>
-    <t>Nazr Mohammed</t>
   </si>
   <si>
     <t>player_season_info</t>
@@ -388,8 +385,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -452,21 +449,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -504,7 +493,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -538,7 +527,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -573,10 +561,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -749,19 +736,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L163"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="29.6640625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -796,78 +780,78 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B3">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F3">
-        <v>1995.724621235355</v>
+        <v>2005.195035749106</v>
       </c>
       <c r="G3">
-        <v>20.682288137511389</v>
+        <v>13.02758933286035</v>
       </c>
       <c r="H3">
-        <v>1947</v>
+        <v>1980</v>
       </c>
       <c r="I3">
-        <v>1980</v>
+        <v>1995</v>
       </c>
       <c r="J3">
-        <v>1999</v>
+        <v>2006</v>
       </c>
       <c r="K3">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="L3">
         <v>2025</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B4">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
         <v>45</v>
       </c>
       <c r="E4">
-        <v>30386</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>24616</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B5">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C5">
-        <v>5266</v>
+        <v>3689</v>
       </c>
       <c r="D5" t="s">
         <v>46</v>
       </c>
       <c r="E5">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B6">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C6">
-        <v>5313</v>
+        <v>3716</v>
       </c>
       <c r="D6" t="s">
         <v>47</v>
@@ -876,18 +860,18 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B7">
-        <v>32586</v>
+        <v>24616</v>
       </c>
       <c r="F7">
-        <v>26.477474989259189</v>
+        <v>26.65262430939227</v>
       </c>
       <c r="G7">
-        <v>3.8545998166572462</v>
+        <v>4.051198795250057</v>
       </c>
       <c r="H7">
         <v>18</v>
@@ -902,32 +886,32 @@
         <v>29</v>
       </c>
       <c r="L7">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B8">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C8">
-        <v>108</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
         <v>48</v>
       </c>
       <c r="E8">
-        <v>2772</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2097</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B9">
-        <v>31410</v>
+        <v>24616</v>
       </c>
       <c r="C9">
         <v>5</v>
@@ -936,50 +920,50 @@
         <v>49</v>
       </c>
       <c r="E9">
-        <v>6606</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+        <v>5125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B10">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F10">
-        <v>48.623198184383241</v>
+        <v>47.48858466038349</v>
       </c>
       <c r="G10">
-        <v>26.615087975149741</v>
+        <v>26.62026950309121</v>
       </c>
       <c r="H10">
         <v>1</v>
       </c>
       <c r="I10">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J10">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K10">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L10">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B11">
-        <v>24451</v>
+        <v>24023</v>
       </c>
       <c r="F11">
-        <v>22.619033986340028</v>
+        <v>22.45385672064272</v>
       </c>
       <c r="G11">
-        <v>28.01768817694424</v>
+        <v>27.88402558272648</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -994,137 +978,137 @@
         <v>42</v>
       </c>
       <c r="L11">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B12">
-        <v>31523</v>
+        <v>24616</v>
       </c>
       <c r="F12">
-        <v>1157.2898835770709</v>
+        <v>1102.884668508287</v>
       </c>
       <c r="G12">
-        <v>925.32966061206923</v>
+        <v>898.533376194927</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>309</v>
+        <v>282</v>
       </c>
       <c r="J12">
-        <v>983</v>
+        <v>915</v>
       </c>
       <c r="K12">
-        <v>1885</v>
+        <v>1798</v>
       </c>
       <c r="L12">
-        <v>3882</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+        <v>3533</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B13">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F13">
-        <v>187.57152057903451</v>
+        <v>177.7025918102048</v>
       </c>
       <c r="G13">
-        <v>184.67987120810881</v>
+        <v>177.1480917816579</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J13">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="K13">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="L13">
-        <v>1597</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B14">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F14">
-        <v>414.42139483530639</v>
+        <v>384.6274780630484</v>
       </c>
       <c r="G14">
-        <v>391.16184434208139</v>
+        <v>370.559922528314</v>
       </c>
       <c r="H14">
         <v>0</v>
       </c>
       <c r="I14">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="J14">
-        <v>301</v>
+        <v>271</v>
       </c>
       <c r="K14">
-        <v>636</v>
+        <v>593</v>
       </c>
       <c r="L14">
-        <v>3159</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2279</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B15">
-        <v>32445</v>
+        <v>24484</v>
       </c>
       <c r="F15">
-        <v>0.43027350901525652</v>
+        <v>0.4398600310406797</v>
       </c>
       <c r="G15">
-        <v>0.10182452356307491</v>
+        <v>0.1021064359919535</v>
       </c>
       <c r="H15">
         <v>0</v>
       </c>
       <c r="I15">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="J15">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="K15">
-        <v>0.48099999999999998</v>
+        <v>0.48825</v>
       </c>
       <c r="L15">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B16">
-        <v>26254</v>
+        <v>24616</v>
       </c>
       <c r="F16">
-        <v>26.428544221832858</v>
+        <v>27.67135196620085</v>
       </c>
       <c r="G16">
-        <v>43.349082275190689</v>
+        <v>44.23624518965004</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -1133,27 +1117,27 @@
         <v>0</v>
       </c>
       <c r="J16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K16">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="L16">
         <v>402</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B17">
-        <v>26253</v>
+        <v>24616</v>
       </c>
       <c r="F17">
-        <v>75.152553993829272</v>
+        <v>78.37926551836205</v>
       </c>
       <c r="G17">
-        <v>115.18249238791201</v>
+        <v>117.3704845304997</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -1162,375 +1146,375 @@
         <v>2</v>
       </c>
       <c r="J17">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K17">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="L17">
         <v>1028</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B18">
-        <v>22032</v>
+        <v>20736</v>
       </c>
       <c r="F18">
-        <v>0.26228603848946991</v>
+        <v>0.2657159529320988</v>
       </c>
       <c r="G18">
-        <v>0.17136152711091299</v>
+        <v>0.1697749444296824</v>
       </c>
       <c r="H18">
         <v>0</v>
       </c>
       <c r="I18">
-        <v>0.154</v>
+        <v>0.167</v>
       </c>
       <c r="J18">
-        <v>0.307</v>
+        <v>0.311</v>
       </c>
       <c r="K18">
-        <v>0.36799999999999999</v>
+        <v>0.37</v>
       </c>
       <c r="L18">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12">
       <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B19">
-        <v>26254</v>
+        <v>24616</v>
       </c>
       <c r="F19">
-        <v>154.43086767730631</v>
+        <v>150.0312398440039</v>
       </c>
       <c r="G19">
-        <v>164.35045375629591</v>
+        <v>160.3960045781875</v>
       </c>
       <c r="H19">
         <v>0</v>
       </c>
       <c r="I19">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J19">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="K19">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="L19">
         <v>1086</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12">
       <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B20">
-        <v>26254</v>
+        <v>24616</v>
       </c>
       <c r="F20">
-        <v>317.05321093928552</v>
+        <v>306.2482125446864</v>
       </c>
       <c r="G20">
-        <v>328.94136709524668</v>
+        <v>318.5622549441325</v>
       </c>
       <c r="H20">
         <v>0</v>
       </c>
       <c r="I20">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J20">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="K20">
-        <v>475</v>
+        <v>457</v>
       </c>
       <c r="L20">
         <v>2213</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B21">
-        <v>26023</v>
+        <v>24395</v>
       </c>
       <c r="F21">
-        <v>0.46736160319717179</v>
+        <v>0.4694487804878049</v>
       </c>
       <c r="G21">
-        <v>0.11009289006878779</v>
+        <v>0.1111386616496463</v>
       </c>
       <c r="H21">
         <v>0</v>
       </c>
       <c r="I21">
-        <v>0.42699999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="J21">
-        <v>0.47299999999999998</v>
+        <v>0.475</v>
       </c>
       <c r="K21">
-        <v>0.51500000000000001</v>
+        <v>0.518</v>
       </c>
       <c r="L21">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B22">
-        <v>26112</v>
+        <v>24484</v>
       </c>
       <c r="F22">
-        <v>0.4723128446691176</v>
+        <v>0.4747831236726025</v>
       </c>
       <c r="G22">
-        <v>0.10561798846438041</v>
+        <v>0.1063436349197005</v>
       </c>
       <c r="H22">
         <v>0</v>
       </c>
       <c r="I22">
-        <v>0.436</v>
+        <v>0.439</v>
       </c>
       <c r="J22">
-        <v>0.48099999999999998</v>
+        <v>0.484</v>
       </c>
       <c r="K22">
-        <v>0.52200000000000002</v>
+        <v>0.524</v>
       </c>
       <c r="L22">
         <v>1.5</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12">
       <c r="A23" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B23">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F23">
-        <v>96.107066184137892</v>
+        <v>86.79732694182646</v>
       </c>
       <c r="G23">
-        <v>110.2918206373095</v>
+        <v>103.4157466297553</v>
       </c>
       <c r="H23">
         <v>0</v>
       </c>
       <c r="I23">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J23">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="K23">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="L23">
-        <v>840</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B24">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F24">
-        <v>128.06805495921</v>
+        <v>114.6895921351966</v>
       </c>
       <c r="G24">
-        <v>141.91696741338311</v>
+        <v>131.7454980686825</v>
       </c>
       <c r="H24">
         <v>0</v>
       </c>
       <c r="I24">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="J24">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="K24">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="L24">
-        <v>1363</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
       <c r="A25" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B25">
-        <v>31272</v>
+        <v>23473</v>
       </c>
       <c r="F25">
-        <v>0.72239712842159121</v>
+        <v>0.7273541941805478</v>
       </c>
       <c r="G25">
-        <v>0.14387529055159121</v>
+        <v>0.1480712462009385</v>
       </c>
       <c r="H25">
         <v>0</v>
       </c>
       <c r="I25">
-        <v>0.66</v>
+        <v>0.667</v>
       </c>
       <c r="J25">
-        <v>0.746</v>
+        <v>0.75</v>
       </c>
       <c r="K25">
-        <v>0.81299999999999994</v>
+        <v>0.819</v>
       </c>
       <c r="L25">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12">
       <c r="A26" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B26">
-        <v>27960</v>
+        <v>24616</v>
       </c>
       <c r="F26">
-        <v>59.224606580829757</v>
+        <v>55.14872440688983</v>
       </c>
       <c r="G26">
-        <v>67.12212058538725</v>
+        <v>62.83593464662353</v>
       </c>
       <c r="H26">
         <v>0</v>
       </c>
       <c r="I26">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J26">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="K26">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L26">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
       <c r="A27" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B27">
-        <v>27960</v>
+        <v>24616</v>
       </c>
       <c r="F27">
-        <v>144.86205293276109</v>
+        <v>139.8024861878453</v>
       </c>
       <c r="G27">
-        <v>146.3008820901878</v>
+        <v>139.5326900407206</v>
       </c>
       <c r="H27">
         <v>0</v>
       </c>
       <c r="I27">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J27">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="K27">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="L27">
-        <v>1111</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
       <c r="A28" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B28">
-        <v>31712</v>
+        <v>24616</v>
       </c>
       <c r="F28">
-        <v>216.23975151362259</v>
+        <v>194.9512105947351</v>
       </c>
       <c r="G28">
-        <v>223.62497805853849</v>
+        <v>196.2916920633748</v>
       </c>
       <c r="H28">
         <v>0</v>
       </c>
       <c r="I28">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="J28">
-        <v>151.5</v>
+        <v>137</v>
       </c>
       <c r="K28">
-        <v>307</v>
+        <v>281</v>
       </c>
       <c r="L28">
-        <v>2149</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
       <c r="A29" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B29">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F29">
-        <v>109.536496350365</v>
+        <v>106.6256499837504</v>
       </c>
       <c r="G29">
-        <v>131.1756438307321</v>
+        <v>132.9362743244503</v>
       </c>
       <c r="H29">
         <v>0</v>
       </c>
       <c r="I29">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J29">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="K29">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="L29">
         <v>1164</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12">
       <c r="A30" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B30">
-        <v>27004</v>
+        <v>24616</v>
       </c>
       <c r="F30">
-        <v>37.765405125166637</v>
+        <v>36.45129184270393</v>
       </c>
       <c r="G30">
-        <v>37.255316779688251</v>
+        <v>36.02421692013997</v>
       </c>
       <c r="H30">
         <v>0</v>
@@ -1539,27 +1523,27 @@
         <v>8</v>
       </c>
       <c r="J30">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K30">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="L30">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
       <c r="A31" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B31">
-        <v>27006</v>
+        <v>24616</v>
       </c>
       <c r="F31">
-        <v>23.2408353699178</v>
+        <v>22.76348716282093</v>
       </c>
       <c r="G31">
-        <v>35.068121400466048</v>
+        <v>34.11322451822389</v>
       </c>
       <c r="H31">
         <v>0</v>
@@ -1577,105 +1561,105 @@
         <v>456</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12">
       <c r="A32" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B32">
-        <v>26970</v>
+        <v>24616</v>
       </c>
       <c r="F32">
-        <v>70.435669262143122</v>
+        <v>67.37077510562236</v>
       </c>
       <c r="G32">
-        <v>67.273855966645243</v>
+        <v>64.6041993767585</v>
       </c>
       <c r="H32">
         <v>0</v>
       </c>
       <c r="I32">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J32">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="K32">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="L32">
         <v>464</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12">
       <c r="A33" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B33">
-        <v>32605</v>
+        <v>24616</v>
       </c>
       <c r="F33">
-        <v>109.20009201042789</v>
+        <v>100.3916964575886</v>
       </c>
       <c r="G33">
-        <v>83.369851635285315</v>
+        <v>78.22141972807761</v>
       </c>
       <c r="H33">
         <v>0</v>
       </c>
       <c r="I33">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J33">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="K33">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="L33">
         <v>386</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12">
       <c r="A34" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B34">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F34">
-        <v>492.53008648714962</v>
+        <v>469.8738625284368</v>
       </c>
       <c r="G34">
-        <v>486.37203341039759</v>
+        <v>471.9510629970359</v>
       </c>
       <c r="H34">
         <v>0</v>
       </c>
       <c r="I34">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="J34">
-        <v>342</v>
+        <v>320</v>
       </c>
       <c r="K34">
-        <v>751</v>
+        <v>721</v>
       </c>
       <c r="L34">
-        <v>4029</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+        <v>3041</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
       <c r="A35" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B35">
-        <v>32601</v>
+        <v>24615</v>
       </c>
       <c r="F35">
-        <v>0.1077267568479495</v>
+        <v>0.1109486085720089</v>
       </c>
       <c r="G35">
-        <v>0.95627831174175904</v>
+        <v>0.9498687936744894</v>
       </c>
       <c r="H35">
         <v>0</v>
@@ -1693,12 +1677,12 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12">
       <c r="A38" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12">
       <c r="B39" s="1" t="s">
         <v>1</v>
       </c>
@@ -1733,61 +1717,61 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B40">
-        <v>3398</v>
+        <v>2897</v>
       </c>
       <c r="F40">
-        <v>1999.7810476751031</v>
+        <v>2005.078702105626</v>
       </c>
       <c r="G40">
-        <v>16.843520415964861</v>
+        <v>11.60312957759442</v>
       </c>
       <c r="H40">
-        <v>1948</v>
+        <v>1980</v>
       </c>
       <c r="I40">
-        <v>1989</v>
+        <v>1996</v>
       </c>
       <c r="J40">
-        <v>2004</v>
+        <v>2007</v>
       </c>
       <c r="K40">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="L40">
         <v>2024</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12">
       <c r="A41" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B41">
-        <v>3398</v>
+        <v>2897</v>
       </c>
       <c r="C41">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D41" t="s">
         <v>57</v>
       </c>
       <c r="E41">
-        <v>1045</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
       <c r="A42" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B42">
-        <v>3398</v>
+        <v>2897</v>
       </c>
       <c r="C42">
-        <v>1025</v>
+        <v>866</v>
       </c>
       <c r="D42" t="s">
         <v>58</v>
@@ -1796,15 +1780,15 @@
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12">
       <c r="A43" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B43">
-        <v>3397</v>
+        <v>2896</v>
       </c>
       <c r="C43">
-        <v>1025</v>
+        <v>866</v>
       </c>
       <c r="D43" t="s">
         <v>59</v>
@@ -1813,18 +1797,18 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12">
       <c r="A44" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B44">
-        <v>3398</v>
+        <v>2897</v>
       </c>
       <c r="F44">
-        <v>26.12654502648617</v>
+        <v>26.15360717984122</v>
       </c>
       <c r="G44">
-        <v>3.836502002109532</v>
+        <v>3.903296029155251</v>
       </c>
       <c r="H44">
         <v>19</v>
@@ -1842,18 +1826,18 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12">
       <c r="A45" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B45">
-        <v>3359</v>
+        <v>2896</v>
       </c>
       <c r="F45">
-        <v>8.1872581125334918</v>
+        <v>7.893301104972376</v>
       </c>
       <c r="G45">
-        <v>20.338806948547809</v>
+        <v>20.25741110501354</v>
       </c>
       <c r="H45">
         <v>0</v>
@@ -1865,27 +1849,27 @@
         <v>1</v>
       </c>
       <c r="K45">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L45">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12">
       <c r="A46" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B46">
-        <v>3375</v>
+        <v>2896</v>
       </c>
       <c r="F46">
-        <v>72.827822222222224</v>
+        <v>76.51101519337017</v>
       </c>
       <c r="G46">
-        <v>168.6071202560419</v>
+        <v>177.0972904932197</v>
       </c>
       <c r="H46">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I46">
         <v>2</v>
@@ -1900,70 +1884,70 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12">
       <c r="A47" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B47">
-        <v>3375</v>
+        <v>2896</v>
       </c>
       <c r="F47">
-        <v>560.44503703703708</v>
+        <v>581.6978591160221</v>
       </c>
       <c r="G47">
-        <v>343.90720700293951</v>
+        <v>339.865026864954</v>
       </c>
       <c r="H47">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="I47">
-        <v>176</v>
+        <v>495</v>
       </c>
       <c r="J47">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="K47">
-        <v>690</v>
+        <v>650</v>
       </c>
       <c r="L47">
         <v>1310</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12">
       <c r="A48" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B48">
-        <v>3375</v>
+        <v>2896</v>
       </c>
       <c r="F48">
-        <v>0.12832740740740739</v>
+        <v>0.1226612569060773</v>
       </c>
       <c r="G48">
-        <v>0.2273916824382346</v>
+        <v>0.2247969774449878</v>
       </c>
       <c r="H48">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="I48">
-        <v>6.0000000000000001E-3</v>
+        <v>0.006</v>
       </c>
       <c r="J48">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="K48">
-        <v>0.128</v>
+        <v>0.112</v>
       </c>
       <c r="L48">
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12">
       <c r="A49" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B49">
-        <v>3398</v>
+        <v>2897</v>
       </c>
       <c r="C49">
         <v>2</v>
@@ -1972,15 +1956,15 @@
         <v>0</v>
       </c>
       <c r="E49">
-        <v>3103</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2680</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12">
       <c r="A52" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12">
       <c r="B53" s="1" t="s">
         <v>1</v>
       </c>
@@ -2015,78 +1999,78 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12">
       <c r="A54" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B54">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F54">
-        <v>1995.724621235355</v>
+        <v>2005.195035749106</v>
       </c>
       <c r="G54">
-        <v>20.682288137511389</v>
+        <v>13.02758933286035</v>
       </c>
       <c r="H54">
-        <v>1947</v>
+        <v>1980</v>
       </c>
       <c r="I54">
-        <v>1980</v>
+        <v>1995</v>
       </c>
       <c r="J54">
-        <v>1999</v>
+        <v>2006</v>
       </c>
       <c r="K54">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="L54">
         <v>2025</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12">
       <c r="A55" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B55">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C55">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D55" t="s">
         <v>45</v>
       </c>
       <c r="E55">
-        <v>30386</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+        <v>24616</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12">
       <c r="A56" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B56">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C56">
-        <v>5266</v>
+        <v>3689</v>
       </c>
       <c r="D56" t="s">
         <v>46</v>
       </c>
       <c r="E56">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12">
       <c r="A57" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B57">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C57">
-        <v>5313</v>
+        <v>3716</v>
       </c>
       <c r="D57" t="s">
         <v>47</v>
@@ -2095,18 +2079,18 @@
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:12">
       <c r="A58" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B58">
-        <v>32586</v>
+        <v>24616</v>
       </c>
       <c r="F58">
-        <v>26.477474989259189</v>
+        <v>26.65262430939227</v>
       </c>
       <c r="G58">
-        <v>3.8545998166572462</v>
+        <v>4.051198795250057</v>
       </c>
       <c r="H58">
         <v>18</v>
@@ -2121,32 +2105,32 @@
         <v>29</v>
       </c>
       <c r="L58">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12">
       <c r="A59" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B59">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C59">
-        <v>108</v>
+        <v>44</v>
       </c>
       <c r="D59" t="s">
         <v>48</v>
       </c>
       <c r="E59">
-        <v>2772</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2097</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12">
       <c r="A60" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B60">
-        <v>31410</v>
+        <v>24616</v>
       </c>
       <c r="C60">
         <v>5</v>
@@ -2155,50 +2139,50 @@
         <v>49</v>
       </c>
       <c r="E60">
-        <v>6606</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+        <v>5125</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12">
       <c r="A61" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B61">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F61">
-        <v>48.623198184383241</v>
+        <v>47.48858466038349</v>
       </c>
       <c r="G61">
-        <v>26.615087975149741</v>
+        <v>26.62026950309121</v>
       </c>
       <c r="H61">
         <v>1</v>
       </c>
       <c r="I61">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J61">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K61">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L61">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12">
       <c r="A62" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B62">
-        <v>24428</v>
+        <v>24023</v>
       </c>
       <c r="F62">
-        <v>22.622318650728669</v>
+        <v>22.45385672064272</v>
       </c>
       <c r="G62">
-        <v>28.021473784870249</v>
+        <v>27.88402558272648</v>
       </c>
       <c r="H62">
         <v>0</v>
@@ -2213,137 +2197,137 @@
         <v>42</v>
       </c>
       <c r="L62">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B63">
-        <v>31523</v>
+        <v>24616</v>
       </c>
       <c r="F63">
-        <v>20.152434730197001</v>
+        <v>19.70303054923627</v>
       </c>
       <c r="G63">
-        <v>10.233139758289489</v>
+        <v>10.04591157552885</v>
       </c>
       <c r="H63">
         <v>0</v>
       </c>
       <c r="I63">
-        <v>11.7</v>
+        <v>11.4</v>
       </c>
       <c r="J63">
-        <v>19.399999999999999</v>
+        <v>19</v>
       </c>
       <c r="K63">
-        <v>28.6</v>
+        <v>27.9</v>
       </c>
       <c r="L63">
-        <v>48.5</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+        <v>44.5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B64">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F64">
-        <v>3.1694258725387958</v>
+        <v>3.063426226844328</v>
       </c>
       <c r="G64">
-        <v>2.3029110256180809</v>
+        <v>2.244522822081189</v>
       </c>
       <c r="H64">
         <v>0</v>
       </c>
       <c r="I64">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="J64">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="K64">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="L64">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B65">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F65">
-        <v>7.1476538060479662</v>
+        <v>6.755248618784531</v>
       </c>
       <c r="G65">
-        <v>4.8280566301555581</v>
+        <v>4.644788805322289</v>
       </c>
       <c r="H65">
         <v>0</v>
       </c>
       <c r="I65">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="J65">
-        <v>6</v>
+        <v>5.6</v>
       </c>
       <c r="K65">
-        <v>10</v>
+        <v>9.4</v>
       </c>
       <c r="L65">
-        <v>39.5</v>
-      </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+        <v>27.8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12">
       <c r="A66" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B66">
-        <v>32445</v>
+        <v>24484</v>
       </c>
       <c r="F66">
-        <v>0.43027350901525652</v>
+        <v>0.4398600310406797</v>
       </c>
       <c r="G66">
-        <v>0.10182452356307491</v>
+        <v>0.1021064359919535</v>
       </c>
       <c r="H66">
         <v>0</v>
       </c>
       <c r="I66">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="J66">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="K66">
-        <v>0.48099999999999998</v>
+        <v>0.48825</v>
       </c>
       <c r="L66">
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:12">
       <c r="A67" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B67">
-        <v>26254</v>
+        <v>24616</v>
       </c>
       <c r="F67">
-        <v>0.47793479088900742</v>
+        <v>0.5012755931101722</v>
       </c>
       <c r="G67">
-        <v>0.66831152426541762</v>
+        <v>0.6802486057357093</v>
       </c>
       <c r="H67">
         <v>0</v>
@@ -2352,7 +2336,7 @@
         <v>0</v>
       </c>
       <c r="J67">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K67">
         <v>0.8</v>
@@ -2361,18 +2345,18 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:12">
       <c r="A68" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B68">
-        <v>26253</v>
+        <v>24616</v>
       </c>
       <c r="F68">
-        <v>1.3913762236696761</v>
+        <v>1.453424601884953</v>
       </c>
       <c r="G68">
-        <v>1.771053109566977</v>
+        <v>1.799637845912231</v>
       </c>
       <c r="H68">
         <v>0</v>
@@ -2381,56 +2365,56 @@
         <v>0</v>
       </c>
       <c r="J68">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="K68">
-        <v>2.2999999999999998</v>
+        <v>2.4</v>
       </c>
       <c r="L68">
         <v>13.2</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:12">
       <c r="A69" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B69">
-        <v>22032</v>
+        <v>20736</v>
       </c>
       <c r="F69">
-        <v>0.26228603848946991</v>
+        <v>0.2657159529320988</v>
       </c>
       <c r="G69">
-        <v>0.17136152711091299</v>
+        <v>0.1697749444296824</v>
       </c>
       <c r="H69">
         <v>0</v>
       </c>
       <c r="I69">
-        <v>0.154</v>
+        <v>0.167</v>
       </c>
       <c r="J69">
-        <v>0.307</v>
+        <v>0.311</v>
       </c>
       <c r="K69">
-        <v>0.36799999999999999</v>
+        <v>0.37</v>
       </c>
       <c r="L69">
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:12">
       <c r="A70" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B70">
-        <v>26254</v>
+        <v>24616</v>
       </c>
       <c r="F70">
-        <v>2.62987354307915</v>
+        <v>2.561801267468313</v>
       </c>
       <c r="G70">
-        <v>2.087607205059101</v>
+        <v>2.048213419974585</v>
       </c>
       <c r="H70">
         <v>0</v>
@@ -2442,198 +2426,198 @@
         <v>2</v>
       </c>
       <c r="K70">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="L70">
         <v>13.2</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:12">
       <c r="A71" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B71">
-        <v>26254</v>
+        <v>24616</v>
       </c>
       <c r="F71">
-        <v>5.477081587567608</v>
+        <v>5.301377153071173</v>
       </c>
       <c r="G71">
-        <v>4.1377532297054511</v>
+        <v>4.021268276334514</v>
       </c>
       <c r="H71">
         <v>0</v>
       </c>
       <c r="I71">
-        <v>2.2999999999999998</v>
+        <v>2.3</v>
       </c>
       <c r="J71">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="K71">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="L71">
-        <v>28.5</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12">
       <c r="A72" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B72">
-        <v>26023</v>
+        <v>24395</v>
       </c>
       <c r="F72">
-        <v>0.46736160319717179</v>
+        <v>0.4694487804878049</v>
       </c>
       <c r="G72">
-        <v>0.11009289006878779</v>
+        <v>0.1111386616496463</v>
       </c>
       <c r="H72">
         <v>0</v>
       </c>
       <c r="I72">
-        <v>0.42699999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="J72">
-        <v>0.47299999999999998</v>
+        <v>0.475</v>
       </c>
       <c r="K72">
-        <v>0.51500000000000001</v>
+        <v>0.518</v>
       </c>
       <c r="L72">
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:12">
       <c r="A73" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B73">
-        <v>26112</v>
+        <v>24484</v>
       </c>
       <c r="F73">
-        <v>0.4723128446691176</v>
+        <v>0.4747831236726025</v>
       </c>
       <c r="G73">
-        <v>0.10561798846438041</v>
+        <v>0.1063436349197005</v>
       </c>
       <c r="H73">
         <v>0</v>
       </c>
       <c r="I73">
-        <v>0.436</v>
+        <v>0.439</v>
       </c>
       <c r="J73">
-        <v>0.48099999999999998</v>
+        <v>0.484</v>
       </c>
       <c r="K73">
-        <v>0.52200000000000002</v>
+        <v>0.524</v>
       </c>
       <c r="L73">
         <v>1.5</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:12">
       <c r="A74" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B74">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F74">
-        <v>1.619438140219591</v>
+        <v>1.484924439389015</v>
       </c>
       <c r="G74">
-        <v>1.4616930406945261</v>
+        <v>1.389992020393045</v>
       </c>
       <c r="H74">
         <v>0</v>
       </c>
       <c r="I74">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="J74">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K74">
-        <v>2.2000000000000002</v>
+        <v>2</v>
       </c>
       <c r="L74">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12">
       <c r="A75" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B75">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F75">
-        <v>2.1816536833711591</v>
+        <v>1.982751056223594</v>
       </c>
       <c r="G75">
-        <v>1.861607074454579</v>
+        <v>1.751176570888355</v>
       </c>
       <c r="H75">
         <v>0</v>
       </c>
       <c r="I75">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="J75">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="K75">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="L75">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12">
       <c r="A76" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B76">
-        <v>31272</v>
+        <v>23473</v>
       </c>
       <c r="F76">
-        <v>0.72239712842159121</v>
+        <v>0.7273541941805478</v>
       </c>
       <c r="G76">
-        <v>0.14387529055159121</v>
+        <v>0.1480712462009385</v>
       </c>
       <c r="H76">
         <v>0</v>
       </c>
       <c r="I76">
-        <v>0.66</v>
+        <v>0.667</v>
       </c>
       <c r="J76">
-        <v>0.746</v>
+        <v>0.75</v>
       </c>
       <c r="K76">
-        <v>0.81299999999999994</v>
+        <v>0.819</v>
       </c>
       <c r="L76">
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:12">
       <c r="A77" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B77">
-        <v>27960</v>
+        <v>24616</v>
       </c>
       <c r="F77">
-        <v>1.03881974248927</v>
+        <v>0.982706369840754</v>
       </c>
       <c r="G77">
-        <v>0.88774708717437389</v>
+        <v>0.8444748941845649</v>
       </c>
       <c r="H77">
         <v>0</v>
@@ -2642,27 +2626,27 @@
         <v>0.4</v>
       </c>
       <c r="J77">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="K77">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="L77">
-        <v>7.2</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12">
       <c r="A78" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B78">
-        <v>27960</v>
+        <v>24616</v>
       </c>
       <c r="F78">
-        <v>2.5315987124463519</v>
+        <v>2.48013080922977</v>
       </c>
       <c r="G78">
-        <v>1.85739505673385</v>
+        <v>1.787502510094779</v>
       </c>
       <c r="H78">
         <v>0</v>
@@ -2674,53 +2658,53 @@
         <v>2.1</v>
       </c>
       <c r="K78">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="L78">
-        <v>13.7</v>
-      </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12">
       <c r="A79" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B79">
-        <v>31712</v>
+        <v>24616</v>
       </c>
       <c r="F79">
-        <v>3.7260658425832491</v>
+        <v>3.461098472538186</v>
       </c>
       <c r="G79">
-        <v>2.8144511121600839</v>
+        <v>2.500271022459904</v>
       </c>
       <c r="H79">
         <v>0</v>
       </c>
       <c r="I79">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="J79">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="K79">
-        <v>4.9000000000000004</v>
+        <v>4.6</v>
       </c>
       <c r="L79">
-        <v>27.2</v>
-      </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12">
       <c r="A80" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B80">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F80">
-        <v>1.875176347911427</v>
+        <v>1.860684107897302</v>
       </c>
       <c r="G80">
-        <v>1.7752484506037289</v>
+        <v>1.832268042162833</v>
       </c>
       <c r="H80">
         <v>0</v>
@@ -2738,18 +2722,18 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:12">
       <c r="A81" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B81">
-        <v>27004</v>
+        <v>24616</v>
       </c>
       <c r="F81">
-        <v>0.66202784772626277</v>
+        <v>0.6487122196945077</v>
       </c>
       <c r="G81">
-        <v>0.47712877365195</v>
+        <v>0.4662529365347882</v>
       </c>
       <c r="H81">
         <v>0</v>
@@ -2764,21 +2748,21 @@
         <v>0.9</v>
       </c>
       <c r="L81">
-        <v>4.0999999999999996</v>
-      </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12">
       <c r="A82" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B82">
-        <v>27006</v>
+        <v>24616</v>
       </c>
       <c r="F82">
-        <v>0.40312893431089392</v>
+        <v>0.4002518687032823</v>
       </c>
       <c r="G82">
-        <v>0.49341772175420701</v>
+        <v>0.4850877377146225</v>
       </c>
       <c r="H82">
         <v>0</v>
@@ -2787,7 +2771,7 @@
         <v>0.1</v>
       </c>
       <c r="J82">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K82">
         <v>0.5</v>
@@ -2796,18 +2780,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:12">
       <c r="A83" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B83">
-        <v>26970</v>
+        <v>24616</v>
       </c>
       <c r="F83">
-        <v>1.251872450871339</v>
+        <v>1.204578323041924</v>
       </c>
       <c r="G83">
-        <v>0.84835049309351107</v>
+        <v>0.8206504463584946</v>
       </c>
       <c r="H83">
         <v>0</v>
@@ -2816,7 +2800,7 @@
         <v>0.6</v>
       </c>
       <c r="J83">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
       <c r="K83">
         <v>1.7</v>
@@ -2825,70 +2809,70 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12">
       <c r="A84" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B84">
-        <v>32605</v>
+        <v>24616</v>
       </c>
       <c r="F84">
-        <v>1.9831988958748661</v>
+        <v>1.856723269418265</v>
       </c>
       <c r="G84">
-        <v>0.91830637670416393</v>
+        <v>0.8709295455812095</v>
       </c>
       <c r="H84">
         <v>0</v>
       </c>
       <c r="I84">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="J84">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="K84">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="L84">
         <v>6</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:12">
       <c r="A85" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B85">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F85">
-        <v>8.3409679200147213</v>
+        <v>8.110940038999026</v>
       </c>
       <c r="G85">
-        <v>6.1064899825129517</v>
+        <v>6.024720163699183</v>
       </c>
       <c r="H85">
         <v>0</v>
       </c>
       <c r="I85">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="J85">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="K85">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="L85">
-        <v>50.4</v>
-      </c>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
+        <v>37.1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12">
       <c r="A88" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:12">
       <c r="B89" s="1" t="s">
         <v>1</v>
       </c>
@@ -2923,7 +2907,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12">
       <c r="A90" s="1" t="s">
         <v>12</v>
       </c>
@@ -2934,7 +2918,7 @@
         <v>2011.930768791736</v>
       </c>
       <c r="G90">
-        <v>8.4407382929821395</v>
+        <v>8.44073829298214</v>
       </c>
       <c r="H90">
         <v>1997</v>
@@ -2952,7 +2936,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:12">
       <c r="A91" s="1" t="s">
         <v>13</v>
       </c>
@@ -2969,7 +2953,7 @@
         <v>17521</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:12">
       <c r="A92" s="1" t="s">
         <v>14</v>
       </c>
@@ -2986,7 +2970,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:12">
       <c r="A93" s="1" t="s">
         <v>15</v>
       </c>
@@ -3003,7 +2987,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:12">
       <c r="A94" s="1" t="s">
         <v>16</v>
       </c>
@@ -3011,10 +2995,10 @@
         <v>17521</v>
       </c>
       <c r="F94">
-        <v>26.658809428685579</v>
+        <v>26.65880942868558</v>
       </c>
       <c r="G94">
-        <v>4.2598285678191203</v>
+        <v>4.25982856781912</v>
       </c>
       <c r="H94">
         <v>18</v>
@@ -3032,7 +3016,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12">
       <c r="A95" s="1" t="s">
         <v>17</v>
       </c>
@@ -3049,7 +3033,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12">
       <c r="A96" s="1" t="s">
         <v>18</v>
       </c>
@@ -3060,13 +3044,13 @@
         <v>5</v>
       </c>
       <c r="D96" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="E96">
         <v>3678</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:12">
       <c r="A97" s="1" t="s">
         <v>19</v>
       </c>
@@ -3074,10 +3058,10 @@
         <v>17521</v>
       </c>
       <c r="F97">
-        <v>45.085040808173048</v>
+        <v>45.08504080817305</v>
       </c>
       <c r="G97">
-        <v>26.043480162458401</v>
+        <v>26.0434801624584</v>
       </c>
       <c r="H97">
         <v>1</v>
@@ -3095,7 +3079,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:12">
       <c r="A98" s="1" t="s">
         <v>20</v>
       </c>
@@ -3124,7 +3108,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:12">
       <c r="A99" s="1" t="s">
         <v>21</v>
       </c>
@@ -3153,7 +3137,7 @@
         <v>3485</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:12">
       <c r="A100" s="1" t="s">
         <v>80</v>
       </c>
@@ -3161,10 +3145,10 @@
         <v>17516</v>
       </c>
       <c r="F100">
-        <v>20.048355788992922</v>
+        <v>20.04835578899292</v>
       </c>
       <c r="G100">
-        <v>36.004292923414397</v>
+        <v>36.0042929234144</v>
       </c>
       <c r="H100">
         <v>0</v>
@@ -3182,7 +3166,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:12">
       <c r="A101" s="1" t="s">
         <v>81</v>
       </c>
@@ -3190,10 +3174,10 @@
         <v>17516</v>
       </c>
       <c r="F101">
-        <v>18.718371774377712</v>
+        <v>18.71837177437771</v>
       </c>
       <c r="G101">
-        <v>29.042036655821342</v>
+        <v>29.04203665582134</v>
       </c>
       <c r="H101">
         <v>0</v>
@@ -3211,7 +3195,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:12">
       <c r="A102" s="1" t="s">
         <v>82</v>
       </c>
@@ -3219,7 +3203,7 @@
         <v>17516</v>
       </c>
       <c r="F102">
-        <v>18.841002511989039</v>
+        <v>18.84100251198904</v>
       </c>
       <c r="G102">
         <v>28.78925977296965</v>
@@ -3240,7 +3224,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:12">
       <c r="A103" s="1" t="s">
         <v>83</v>
       </c>
@@ -3269,7 +3253,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:12">
       <c r="A104" s="1" t="s">
         <v>84</v>
       </c>
@@ -3277,10 +3261,10 @@
         <v>17516</v>
       </c>
       <c r="F104">
-        <v>22.438912993834212</v>
+        <v>22.43891299383421</v>
       </c>
       <c r="G104">
-        <v>37.036329879063913</v>
+        <v>37.03632987906391</v>
       </c>
       <c r="H104">
         <v>0</v>
@@ -3298,7 +3282,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:12">
       <c r="A105" s="1" t="s">
         <v>85</v>
       </c>
@@ -3306,10 +3290,10 @@
         <v>17512</v>
       </c>
       <c r="F105">
-        <v>-2.7510678391959802</v>
+        <v>-2.75106783919598</v>
       </c>
       <c r="G105">
-        <v>14.894267638904219</v>
+        <v>14.89426763890422</v>
       </c>
       <c r="H105">
         <v>-300</v>
@@ -3327,7 +3311,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:12">
       <c r="A106" s="1" t="s">
         <v>86</v>
       </c>
@@ -3335,10 +3319,10 @@
         <v>17512</v>
       </c>
       <c r="F106">
-        <v>-2.1789915486523519</v>
+        <v>-2.178991548652352</v>
       </c>
       <c r="G106">
-        <v>15.103878030953201</v>
+        <v>15.1038780309532</v>
       </c>
       <c r="H106">
         <v>-303</v>
@@ -3353,10 +3337,10 @@
         <v>3.6</v>
       </c>
       <c r="L106">
-        <v>308.10000000000002</v>
-      </c>
-    </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
+        <v>308.1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12">
       <c r="A107" s="1" t="s">
         <v>87</v>
       </c>
@@ -3364,10 +3348,10 @@
         <v>17521</v>
       </c>
       <c r="F107">
-        <v>27.858113121397182</v>
+        <v>27.85811312139718</v>
       </c>
       <c r="G107">
-        <v>31.316882099077532</v>
+        <v>31.31688209907753</v>
       </c>
       <c r="H107">
         <v>0</v>
@@ -3385,7 +3369,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:12">
       <c r="A108" s="1" t="s">
         <v>88</v>
       </c>
@@ -3393,7 +3377,7 @@
         <v>17521</v>
       </c>
       <c r="F108">
-        <v>15.609725472290391</v>
+        <v>15.60972547229039</v>
       </c>
       <c r="G108">
         <v>16.94394347483145</v>
@@ -3414,7 +3398,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:12">
       <c r="A109" s="1" t="s">
         <v>89</v>
       </c>
@@ -3422,10 +3406,10 @@
         <v>17521</v>
       </c>
       <c r="F109">
-        <v>42.914217225044233</v>
+        <v>42.91421722504423</v>
       </c>
       <c r="G109">
-        <v>35.254147452250237</v>
+        <v>35.25414745225024</v>
       </c>
       <c r="H109">
         <v>0</v>
@@ -3443,7 +3427,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:12">
       <c r="A110" s="1" t="s">
         <v>90</v>
       </c>
@@ -3472,7 +3456,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:12">
       <c r="A111" s="1" t="s">
         <v>91</v>
       </c>
@@ -3480,10 +3464,10 @@
         <v>17521</v>
       </c>
       <c r="F111">
-        <v>42.244392443353689</v>
+        <v>42.24439244335369</v>
       </c>
       <c r="G111">
-        <v>51.578124628154093</v>
+        <v>51.57812462815409</v>
       </c>
       <c r="H111">
         <v>0</v>
@@ -3501,7 +3485,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:12">
       <c r="A112" s="1" t="s">
         <v>92</v>
       </c>
@@ -3509,10 +3493,10 @@
         <v>12707</v>
       </c>
       <c r="F112">
-        <v>6.5788148264735966</v>
+        <v>6.578814826473597</v>
       </c>
       <c r="G112">
-        <v>8.3839463844373441</v>
+        <v>8.383946384437344</v>
       </c>
       <c r="H112">
         <v>0</v>
@@ -3530,7 +3514,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:12">
       <c r="A113" s="1" t="s">
         <v>93</v>
       </c>
@@ -3538,10 +3522,10 @@
         <v>17521</v>
       </c>
       <c r="F113">
-        <v>223.50202614006051</v>
+        <v>223.5020261400605</v>
       </c>
       <c r="G113">
-        <v>280.76345710540818</v>
+        <v>280.7634571054082</v>
       </c>
       <c r="H113">
         <v>0</v>
@@ -3559,7 +3543,7 @@
         <v>2179</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:12">
       <c r="A114" s="1" t="s">
         <v>94</v>
       </c>
@@ -3567,10 +3551,10 @@
         <v>17521</v>
       </c>
       <c r="F114">
-        <v>9.3614519719194114</v>
+        <v>9.361451971919411</v>
       </c>
       <c r="G114">
-        <v>12.299464304753061</v>
+        <v>12.29946430475306</v>
       </c>
       <c r="H114">
         <v>0</v>
@@ -3588,7 +3572,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:12">
       <c r="A115" s="1" t="s">
         <v>95</v>
       </c>
@@ -3596,10 +3580,10 @@
         <v>17521</v>
       </c>
       <c r="F115">
-        <v>21.099765995091609</v>
+        <v>21.09976599509161</v>
       </c>
       <c r="G115">
-        <v>21.801566710176999</v>
+        <v>21.801566710177</v>
       </c>
       <c r="H115">
         <v>0</v>
@@ -3617,12 +3601,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12">
       <c r="B119" s="1" t="s">
         <v>1</v>
       </c>
@@ -3657,78 +3641,78 @@
         <v>11</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:12">
       <c r="A120" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B120">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F120">
-        <v>1995.724621235355</v>
+        <v>2005.195035749106</v>
       </c>
       <c r="G120">
-        <v>20.682288137511389</v>
+        <v>13.02758933286035</v>
       </c>
       <c r="H120">
-        <v>1947</v>
+        <v>1980</v>
       </c>
       <c r="I120">
-        <v>1980</v>
+        <v>1995</v>
       </c>
       <c r="J120">
-        <v>1999</v>
+        <v>2006</v>
       </c>
       <c r="K120">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="L120">
         <v>2025</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:12">
       <c r="A121" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B121">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C121">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D121" t="s">
         <v>45</v>
       </c>
       <c r="E121">
-        <v>30386</v>
-      </c>
-    </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
+        <v>24616</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12">
       <c r="A122" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B122">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C122">
-        <v>5266</v>
+        <v>3689</v>
       </c>
       <c r="D122" t="s">
         <v>46</v>
       </c>
       <c r="E122">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12">
       <c r="A123" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B123">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C123">
-        <v>5313</v>
+        <v>3716</v>
       </c>
       <c r="D123" t="s">
         <v>47</v>
@@ -3737,18 +3721,18 @@
         <v>28</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:12">
       <c r="A124" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B124">
-        <v>32586</v>
+        <v>24616</v>
       </c>
       <c r="F124">
-        <v>26.477474989259189</v>
+        <v>26.65262430939227</v>
       </c>
       <c r="G124">
-        <v>3.8545998166572462</v>
+        <v>4.051198795250057</v>
       </c>
       <c r="H124">
         <v>18</v>
@@ -3763,32 +3747,32 @@
         <v>29</v>
       </c>
       <c r="L124">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12">
       <c r="A125" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B125">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="C125">
-        <v>108</v>
+        <v>44</v>
       </c>
       <c r="D125" t="s">
         <v>48</v>
       </c>
       <c r="E125">
-        <v>2772</v>
-      </c>
-    </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.2">
+        <v>2097</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12">
       <c r="A126" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B126">
-        <v>31410</v>
+        <v>24616</v>
       </c>
       <c r="C126">
         <v>5</v>
@@ -3797,21 +3781,21 @@
         <v>49</v>
       </c>
       <c r="E126">
-        <v>6606</v>
-      </c>
-    </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.2">
+        <v>5125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12">
       <c r="A127" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B127">
-        <v>32606</v>
+        <v>24616</v>
       </c>
       <c r="F127">
-        <v>4.9809237563638593</v>
+        <v>5.409002274943126</v>
       </c>
       <c r="G127">
-        <v>3.7360552341561402</v>
+        <v>3.906141172860314</v>
       </c>
       <c r="H127">
         <v>1</v>
@@ -3823,18 +3807,18 @@
         <v>4</v>
       </c>
       <c r="K127">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L127">
         <v>22</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:12">
       <c r="A130" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12">
       <c r="B131" s="1" t="s">
         <v>1</v>
       </c>
@@ -3869,7 +3853,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:12">
       <c r="A132" s="1" t="s">
         <v>12</v>
       </c>
@@ -3880,7 +3864,7 @@
         <v>2011.930768791736</v>
       </c>
       <c r="G132">
-        <v>8.4407382929821395</v>
+        <v>8.44073829298214</v>
       </c>
       <c r="H132">
         <v>1997</v>
@@ -3898,7 +3882,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:12">
       <c r="A133" s="1" t="s">
         <v>13</v>
       </c>
@@ -3915,7 +3899,7 @@
         <v>17521</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:12">
       <c r="A134" s="1" t="s">
         <v>14</v>
       </c>
@@ -3932,7 +3916,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:12">
       <c r="A135" s="1" t="s">
         <v>15</v>
       </c>
@@ -3949,7 +3933,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:12">
       <c r="A136" s="1" t="s">
         <v>16</v>
       </c>
@@ -3957,10 +3941,10 @@
         <v>17521</v>
       </c>
       <c r="F136">
-        <v>26.658809428685579</v>
+        <v>26.65880942868558</v>
       </c>
       <c r="G136">
-        <v>4.2598285678191203</v>
+        <v>4.25982856781912</v>
       </c>
       <c r="H136">
         <v>18</v>
@@ -3978,7 +3962,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:12">
       <c r="A137" s="1" t="s">
         <v>17</v>
       </c>
@@ -3995,7 +3979,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:12">
       <c r="A138" s="1" t="s">
         <v>18</v>
       </c>
@@ -4006,13 +3990,13 @@
         <v>5</v>
       </c>
       <c r="D138" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="E138">
         <v>3678</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:12">
       <c r="A139" s="1" t="s">
         <v>19</v>
       </c>
@@ -4020,10 +4004,10 @@
         <v>17521</v>
       </c>
       <c r="F139">
-        <v>45.085040808173048</v>
+        <v>45.08504080817305</v>
       </c>
       <c r="G139">
-        <v>26.043480162458401</v>
+        <v>26.0434801624584</v>
       </c>
       <c r="H139">
         <v>1</v>
@@ -4041,7 +4025,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:12">
       <c r="A140" s="1" t="s">
         <v>20</v>
       </c>
@@ -4070,7 +4054,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:12">
       <c r="A141" s="1" t="s">
         <v>21</v>
       </c>
@@ -4099,7 +4083,7 @@
         <v>3485</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:12">
       <c r="A142" s="1" t="s">
         <v>24</v>
       </c>
@@ -4107,30 +4091,30 @@
         <v>17414</v>
       </c>
       <c r="F142">
-        <v>0.43480722407258532</v>
+        <v>0.4348072240725853</v>
       </c>
       <c r="G142">
-        <v>0.10582133496212159</v>
+        <v>0.1058213349621216</v>
       </c>
       <c r="H142">
         <v>0</v>
       </c>
       <c r="I142">
-        <v>0.39500000000000002</v>
+        <v>0.395</v>
       </c>
       <c r="J142">
         <v>0.437</v>
       </c>
       <c r="K142">
-        <v>0.48199999999999998</v>
+        <v>0.482</v>
       </c>
       <c r="L142">
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:12">
       <c r="A143" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B143">
         <v>17414</v>
@@ -4139,7 +4123,7 @@
         <v>12.59656023888825</v>
       </c>
       <c r="G143">
-        <v>5.0080154208109304</v>
+        <v>5.00801542081093</v>
       </c>
       <c r="H143">
         <v>0</v>
@@ -4157,15 +4141,15 @@
         <v>45.3</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:12">
       <c r="A144" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B144">
         <v>17414</v>
       </c>
       <c r="F144">
-        <v>0.73127139083496029</v>
+        <v>0.7312713908349603</v>
       </c>
       <c r="G144">
         <v>0.2270427035060836</v>
@@ -4174,27 +4158,27 @@
         <v>0</v>
       </c>
       <c r="I144">
-        <v>0.56599999999999995</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="J144">
-        <v>0.73699999999999999</v>
+        <v>0.737</v>
       </c>
       <c r="K144">
-        <v>0.97399999999999998</v>
+        <v>0.974</v>
       </c>
       <c r="L144">
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:12">
       <c r="A145" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B145">
         <v>17414</v>
       </c>
       <c r="F145">
-        <v>0.30274422878144019</v>
+        <v>0.3027442287814402</v>
       </c>
       <c r="G145">
         <v>0.181145853333819</v>
@@ -4203,39 +4187,39 @@
         <v>0</v>
       </c>
       <c r="I145">
-        <v>0.17499999999999999</v>
+        <v>0.175</v>
       </c>
       <c r="J145">
-        <v>0.27100000000000002</v>
+        <v>0.271</v>
       </c>
       <c r="K145">
-        <v>0.39600000000000002</v>
+        <v>0.396</v>
       </c>
       <c r="L145">
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:12">
       <c r="A146" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B146">
         <v>17414</v>
       </c>
       <c r="F146">
-        <v>0.16508050993453549</v>
+        <v>0.1650805099345355</v>
       </c>
       <c r="G146">
-        <v>0.11660362217711059</v>
+        <v>0.1166036221771106</v>
       </c>
       <c r="H146">
         <v>0</v>
       </c>
       <c r="I146">
-        <v>8.5000000000000006E-2</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="J146">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="K146">
         <v>0.222</v>
@@ -4244,38 +4228,38 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:12">
       <c r="A147" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B147">
         <v>17414</v>
       </c>
       <c r="F147">
-        <v>0.10608929596876079</v>
+        <v>0.1060892959687608</v>
       </c>
       <c r="G147">
-        <v>8.7389685371503101E-2</v>
+        <v>0.0873896853715031</v>
       </c>
       <c r="H147">
         <v>0</v>
       </c>
       <c r="I147">
-        <v>5.0999999999999997E-2</v>
+        <v>0.051</v>
       </c>
       <c r="J147">
-        <v>9.0999999999999998E-2</v>
+        <v>0.091</v>
       </c>
       <c r="K147">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="L147">
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:12">
       <c r="A148" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B148">
         <v>17414</v>
@@ -4284,45 +4268,45 @@
         <v>0.1572340645457678</v>
       </c>
       <c r="G148">
-        <v>0.13623012341531349</v>
+        <v>0.1362301234153135</v>
       </c>
       <c r="H148">
         <v>0</v>
       </c>
       <c r="I148">
-        <v>4.5999999999999999E-2</v>
+        <v>0.046</v>
       </c>
       <c r="J148">
         <v>0.13</v>
       </c>
       <c r="K148">
-        <v>0.23899999999999999</v>
+        <v>0.239</v>
       </c>
       <c r="L148">
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:12">
       <c r="A149" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B149">
         <v>17414</v>
       </c>
       <c r="F149">
-        <v>0.26873331801998401</v>
+        <v>0.268733318019984</v>
       </c>
       <c r="G149">
-        <v>0.22704307003240121</v>
+        <v>0.2270430700324012</v>
       </c>
       <c r="H149">
         <v>0</v>
       </c>
       <c r="I149">
-        <v>2.5999999999999999E-2</v>
+        <v>0.026</v>
       </c>
       <c r="J149">
-        <v>0.26300000000000001</v>
+        <v>0.263</v>
       </c>
       <c r="K149">
         <v>0.434</v>
@@ -4331,154 +4315,154 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:12">
       <c r="A150" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B150">
         <v>17331</v>
       </c>
       <c r="F150">
-        <v>0.47163406612428599</v>
+        <v>0.471634066124286</v>
       </c>
       <c r="G150">
-        <v>0.11767036347409079</v>
+        <v>0.1176703634740908</v>
       </c>
       <c r="H150">
         <v>0</v>
       </c>
       <c r="I150">
-        <v>0.42699999999999999</v>
+        <v>0.427</v>
       </c>
       <c r="J150">
-        <v>0.47499999999999998</v>
+        <v>0.475</v>
       </c>
       <c r="K150">
-        <v>0.52500000000000002</v>
+        <v>0.525</v>
       </c>
       <c r="L150">
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:12">
       <c r="A151" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B151">
         <v>16928</v>
       </c>
       <c r="F151">
-        <v>0.60906250000000006</v>
+        <v>0.6090625000000001</v>
       </c>
       <c r="G151">
-        <v>0.15123116372965961</v>
+        <v>0.1512311637296596</v>
       </c>
       <c r="H151">
         <v>0</v>
       </c>
       <c r="I151">
-        <v>0.54400000000000004</v>
+        <v>0.544</v>
       </c>
       <c r="J151">
-        <v>0.61799999999999999</v>
+        <v>0.618</v>
       </c>
       <c r="K151">
-        <v>0.68400000000000005</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="L151">
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:12">
       <c r="A152" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B152">
         <v>16590</v>
       </c>
       <c r="F152">
-        <v>0.36660578661844478</v>
+        <v>0.3666057866184448</v>
       </c>
       <c r="G152">
-        <v>0.16822240807587591</v>
+        <v>0.1682224080758759</v>
       </c>
       <c r="H152">
         <v>0</v>
       </c>
       <c r="I152">
-        <v>0.29399999999999998</v>
+        <v>0.294</v>
       </c>
       <c r="J152">
         <v>0.379</v>
       </c>
       <c r="K152">
-        <v>0.45100000000000001</v>
+        <v>0.451</v>
       </c>
       <c r="L152">
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:12">
       <c r="A153" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B153">
         <v>16108</v>
       </c>
       <c r="F153">
-        <v>0.35681152222498141</v>
+        <v>0.3568115222249814</v>
       </c>
       <c r="G153">
-        <v>0.18550521221104321</v>
+        <v>0.1855052122110432</v>
       </c>
       <c r="H153">
         <v>0</v>
       </c>
       <c r="I153">
-        <v>0.27300000000000002</v>
+        <v>0.273</v>
       </c>
       <c r="J153">
         <v>0.37</v>
       </c>
       <c r="K153">
-        <v>0.44900000000000001</v>
+        <v>0.449</v>
       </c>
       <c r="L153">
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:12">
       <c r="A154" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B154">
         <v>15895</v>
       </c>
       <c r="F154">
-        <v>0.36091947153192833</v>
+        <v>0.3609194715319283</v>
       </c>
       <c r="G154">
-        <v>0.18146696330761591</v>
+        <v>0.1814669633076159</v>
       </c>
       <c r="H154">
         <v>0</v>
       </c>
       <c r="I154">
-        <v>0.29299999999999998</v>
+        <v>0.293</v>
       </c>
       <c r="J154">
         <v>0.379</v>
       </c>
       <c r="K154">
-        <v>0.44400000000000001</v>
+        <v>0.444</v>
       </c>
       <c r="L154">
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:12">
       <c r="A155" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B155">
         <v>15063</v>
@@ -4487,13 +4471,13 @@
         <v>0.2893926176724424</v>
       </c>
       <c r="G155">
-        <v>0.15771731451737181</v>
+        <v>0.1577173145173718</v>
       </c>
       <c r="H155">
         <v>0</v>
       </c>
       <c r="I155">
-        <v>0.23100000000000001</v>
+        <v>0.231</v>
       </c>
       <c r="J155">
         <v>0.33</v>
@@ -4505,44 +4489,44 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:12">
       <c r="A156" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B156">
         <v>17027</v>
       </c>
       <c r="F156">
-        <v>0.55191390145063712</v>
+        <v>0.5519139014506371</v>
       </c>
       <c r="G156">
-        <v>0.20933592648525379</v>
+        <v>0.2093359264852538</v>
       </c>
       <c r="H156">
         <v>0</v>
       </c>
       <c r="I156">
-        <v>0.41499999999999998</v>
+        <v>0.415</v>
       </c>
       <c r="J156">
-        <v>0.58099999999999996</v>
+        <v>0.581</v>
       </c>
       <c r="K156">
-        <v>0.69499999999999995</v>
+        <v>0.695</v>
       </c>
       <c r="L156">
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:12">
       <c r="A157" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B157">
         <v>12845</v>
       </c>
       <c r="F157">
-        <v>0.86209824834565985</v>
+        <v>0.8620982483456598</v>
       </c>
       <c r="G157">
         <v>0.1865342772623467</v>
@@ -4554,7 +4538,7 @@
         <v>0.8</v>
       </c>
       <c r="J157">
-        <v>0.93200000000000005</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="K157">
         <v>1</v>
@@ -4563,18 +4547,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:12">
       <c r="A158" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B158">
         <v>17414</v>
       </c>
       <c r="F158">
-        <v>5.7205409440679908E-2</v>
+        <v>0.05720540944067991</v>
       </c>
       <c r="G158">
-        <v>8.330520378445902E-2</v>
+        <v>0.08330520378445902</v>
       </c>
       <c r="H158">
         <v>0</v>
@@ -4583,18 +4567,18 @@
         <v>0</v>
       </c>
       <c r="J158">
-        <v>2.7E-2</v>
+        <v>0.027</v>
       </c>
       <c r="K158">
-        <v>7.6999999999999999E-2</v>
+        <v>0.077</v>
       </c>
       <c r="L158">
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:12">
       <c r="A159" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B159">
         <v>17521</v>
@@ -4621,18 +4605,18 @@
         <v>306</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:12">
       <c r="A160" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B160">
         <v>15063</v>
       </c>
       <c r="F160">
-        <v>0.25579818097324569</v>
+        <v>0.2557981809732457</v>
       </c>
       <c r="G160">
-        <v>0.20678365774263921</v>
+        <v>0.2067836577426392</v>
       </c>
       <c r="H160">
         <v>0</v>
@@ -4644,24 +4628,24 @@
         <v>0.224</v>
       </c>
       <c r="K160">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="L160">
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:12">
       <c r="A161" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B161">
         <v>12929</v>
       </c>
       <c r="F161">
-        <v>0.34242176502436378</v>
+        <v>0.3424217650243638</v>
       </c>
       <c r="G161">
-        <v>0.20187036386089771</v>
+        <v>0.2018703638608977</v>
       </c>
       <c r="H161">
         <v>0</v>
@@ -4670,24 +4654,24 @@
         <v>0.25</v>
       </c>
       <c r="J161">
-        <v>0.36399999999999999</v>
+        <v>0.364</v>
       </c>
       <c r="K161">
-        <v>0.44400000000000001</v>
+        <v>0.444</v>
       </c>
       <c r="L161">
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:12">
       <c r="A162" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B162">
         <v>17521</v>
       </c>
       <c r="F162">
-        <v>0.70429769990297353</v>
+        <v>0.7042976999029735</v>
       </c>
       <c r="G162">
         <v>1.354743197606481</v>
@@ -4708,18 +4692,18 @@
         <v>22</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:12">
       <c r="A163" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B163">
         <v>17521</v>
       </c>
       <c r="F163">
-        <v>1.797842588893328E-2</v>
+        <v>0.01797842588893328</v>
       </c>
       <c r="G163">
-        <v>0.13917089701380481</v>
+        <v>0.1391708970138048</v>
       </c>
       <c r="H163">
         <v>0</v>

</xml_diff>